<commit_message>
Verify BR MU FM flight schedules
</commit_message>
<xml_diff>
--- a/routes.xlsx
+++ b/routes.xlsx
@@ -14,7 +14,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$B$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Routes'!$A$1:$P$101</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Routes'!$A$1:$P$102</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Source Checks'!$A$1:$E$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Integrity Checks'!$A$1:$D$27</definedName>
   </definedNames>
@@ -156,8 +156,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Routes" displayName="Routes" ref="A1:P101" headerRowCount="1">
-  <autoFilter ref="A1:P101"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Routes" displayName="Routes" ref="A1:P102" headerRowCount="1">
+  <autoFilter ref="A1:P102"/>
   <tableColumns count="16">
     <tableColumn id="1" name="airline"/>
     <tableColumn id="2" name="flight_number"/>
@@ -522,7 +522,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="3">
@@ -532,7 +532,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>53</v>
+        <v>101</v>
       </c>
     </row>
     <row r="4">
@@ -542,7 +542,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>47</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -584,7 +584,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P101"/>
+  <dimension ref="A1:P102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -4884,22 +4884,22 @@
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>EVA Air official timetable page plus route-level cross-check</t>
+          <t>EVA Air official timetable page, cross-checked with FlightMapper/Flight.info</t>
         </is>
       </c>
       <c r="N55" t="inlineStr">
         <is>
-          <t>https://booking.evaair.com/flyeva/eva/b2c/flight-schedules.aspx?lang=en-global</t>
+          <t>https://info.flightmapper.net/flight/EVA_Air_BR_809</t>
         </is>
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="P55" t="inlineStr">
         <is>
-          <t>Cross-checked with FlightMapper route page; final EVA query should be re-run.</t>
+          <t>Confirmed for 2026 summer public schedule.</t>
         </is>
       </c>
     </row>
@@ -4966,22 +4966,22 @@
       </c>
       <c r="M56" t="inlineStr">
         <is>
-          <t>EVA Air official timetable page plus route-level cross-check</t>
+          <t>EVA Air official timetable page, cross-checked with FlightMapper/Flight.info</t>
         </is>
       </c>
       <c r="N56" t="inlineStr">
         <is>
-          <t>https://booking.evaair.com/flyeva/eva/b2c/flight-schedules.aspx?lang=en-global</t>
+          <t>https://info.flightmapper.net/flight/EVA_Air_BR_851</t>
         </is>
       </c>
       <c r="O56" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="P56" t="inlineStr">
         <is>
-          <t>Cross-checked with FlightMapper route page; final EVA query should be re-run.</t>
+          <t>Confirmed for 2026 summer public schedule.</t>
         </is>
       </c>
     </row>
@@ -5048,22 +5048,22 @@
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>EVA Air official timetable page plus route-level cross-check</t>
+          <t>EVA Air official timetable page, cross-checked with FlightMapper/Flight.info</t>
         </is>
       </c>
       <c r="N57" t="inlineStr">
         <is>
-          <t>https://booking.evaair.com/flyeva/eva/b2c/flight-schedules.aspx?lang=en-global</t>
+          <t>https://info.flightmapper.net/flight/EVA_Air_BR_857</t>
         </is>
       </c>
       <c r="O57" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="P57" t="inlineStr">
         <is>
-          <t>Cross-checked with FlightMapper route page; final EVA query should be re-run.</t>
+          <t>Confirmed for 2026 summer public schedule.</t>
         </is>
       </c>
     </row>
@@ -5125,27 +5125,27 @@
       </c>
       <c r="L58" t="inlineStr">
         <is>
-          <t>321</t>
+          <t>789</t>
         </is>
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>EVA Air official timetable page plus route-level cross-check</t>
+          <t>EVA Air official timetable page, cross-checked with FlightMapper/Flight.info</t>
         </is>
       </c>
       <c r="N58" t="inlineStr">
         <is>
-          <t>https://booking.evaair.com/flyeva/eva/b2c/flight-schedules.aspx?lang=en-global</t>
+          <t>https://www.flight.info/BR867</t>
         </is>
       </c>
       <c r="O58" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="P58" t="inlineStr">
         <is>
-          <t>Cross-checked with FlightMapper route page; final EVA query should be re-run.</t>
+          <t>Confirmed for 2026 summer public schedule.</t>
         </is>
       </c>
     </row>
@@ -5212,22 +5212,22 @@
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>EVA Air official timetable page plus route-level cross-check</t>
+          <t>EVA Air official timetable page, cross-checked with FlightMapper/Flight.info</t>
         </is>
       </c>
       <c r="N59" t="inlineStr">
         <is>
-          <t>https://booking.evaair.com/flyeva/eva/b2c/flight-schedules.aspx?lang=en-global</t>
+          <t>https://info.flightmapper.net/flight/EVA_Air_BR_869</t>
         </is>
       </c>
       <c r="O59" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="P59" t="inlineStr">
         <is>
-          <t>Cross-checked with FlightMapper route page; final EVA query should be re-run.</t>
+          <t>Confirmed for 2026 summer public schedule.</t>
         </is>
       </c>
     </row>
@@ -5294,22 +5294,22 @@
       </c>
       <c r="M60" t="inlineStr">
         <is>
-          <t>EVA Air official timetable page plus route-level cross-check</t>
+          <t>EVA Air official timetable page, cross-checked with FlightMapper/Flight.info</t>
         </is>
       </c>
       <c r="N60" t="inlineStr">
         <is>
-          <t>https://booking.evaair.com/flyeva/eva/b2c/flight-schedules.aspx?lang=en-global</t>
+          <t>https://info.flightmapper.net/flight/EVA_Air_BR_871</t>
         </is>
       </c>
       <c r="O60" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="P60" t="inlineStr">
         <is>
-          <t>Cross-checked with FlightMapper route page; final EVA query should be re-run.</t>
+          <t>Confirmed for 2026 summer public schedule.</t>
         </is>
       </c>
     </row>
@@ -5376,22 +5376,22 @@
       </c>
       <c r="M61" t="inlineStr">
         <is>
-          <t>EVA Air official timetable page plus route-level cross-check</t>
+          <t>EVA Air official timetable page, cross-checked with FlightMapper/Flight.info</t>
         </is>
       </c>
       <c r="N61" t="inlineStr">
         <is>
-          <t>https://booking.evaair.com/flyeva/eva/b2c/flight-schedules.aspx?lang=en-global</t>
+          <t>https://info.flightmapper.net/flight/EVA_Air_BR_801</t>
         </is>
       </c>
       <c r="O61" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="P61" t="inlineStr">
         <is>
-          <t>Cross-checked with FlightMapper route page; final EVA query should be re-run.</t>
+          <t>Confirmed for 2026 summer public schedule.</t>
         </is>
       </c>
     </row>
@@ -5458,22 +5458,22 @@
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>EVA Air official timetable page plus route-level cross-check</t>
+          <t>EVA Air official timetable page, cross-checked with FlightMapper/Flight.info</t>
         </is>
       </c>
       <c r="N62" t="inlineStr">
         <is>
-          <t>https://booking.evaair.com/flyeva/eva/b2c/flight-schedules.aspx?lang=en-global</t>
+          <t>https://info.flightmapper.net/flight/EVA_Air_BR_806</t>
         </is>
       </c>
       <c r="O62" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="P62" t="inlineStr">
         <is>
-          <t>Cross-checked with FlightMapper route page; final EVA query should be re-run.</t>
+          <t>Confirmed for 2026 summer public schedule.</t>
         </is>
       </c>
     </row>
@@ -5540,22 +5540,22 @@
       </c>
       <c r="M63" t="inlineStr">
         <is>
-          <t>EVA Air official timetable page plus route-level cross-check</t>
+          <t>EVA Air official timetable page, cross-checked with FlightMapper/Flight.info</t>
         </is>
       </c>
       <c r="N63" t="inlineStr">
         <is>
-          <t>https://booking.evaair.com/flyeva/eva/b2c/flight-schedules.aspx?lang=en-global</t>
+          <t>https://www.flight.info/BR829</t>
         </is>
       </c>
       <c r="O63" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>Cross-checked with FlightMapper route page; final EVA query should be re-run.</t>
+          <t>Confirmed for 2026 summer public schedule.</t>
         </is>
       </c>
     </row>
@@ -5597,12 +5597,12 @@
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>11:35</t>
+          <t>11:45</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>13:15</t>
         </is>
       </c>
       <c r="J64" t="inlineStr">
@@ -5622,22 +5622,22 @@
       </c>
       <c r="M64" t="inlineStr">
         <is>
-          <t>EVA Air official timetable page plus route-level cross-check</t>
+          <t>EVA Air official timetable page, cross-checked with FlightMapper/Flight.info</t>
         </is>
       </c>
       <c r="N64" t="inlineStr">
         <is>
-          <t>https://booking.evaair.com/flyeva/eva/b2c/flight-schedules.aspx?lang=en-global</t>
+          <t>https://www.flight.info/BR830</t>
         </is>
       </c>
       <c r="O64" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>Cross-checked with FlightMapper route page; final EVA query should be re-run.</t>
+          <t>Confirmed for 2026 summer public schedule.</t>
         </is>
       </c>
     </row>
@@ -5704,22 +5704,22 @@
       </c>
       <c r="M65" t="inlineStr">
         <is>
-          <t>EVA Air official timetable page plus route-level cross-check</t>
+          <t>EVA Air official timetable page, cross-checked with FlightMapper/Flight.info</t>
         </is>
       </c>
       <c r="N65" t="inlineStr">
         <is>
-          <t>https://booking.evaair.com/flyeva/eva/b2c/flight-schedules.aspx?lang=en-global</t>
+          <t>https://info.flightmapper.net/flight/EVA_Air_BR_716</t>
         </is>
       </c>
       <c r="O65" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="P65" t="inlineStr">
         <is>
-          <t>Cross-checked with FlightMapper route page; final EVA query should be re-run.</t>
+          <t>Confirmed for 2026 summer public schedule.</t>
         </is>
       </c>
     </row>
@@ -5786,22 +5786,22 @@
       </c>
       <c r="M66" t="inlineStr">
         <is>
-          <t>EVA Air official timetable page plus route-level cross-check</t>
+          <t>EVA Air official timetable page, cross-checked with FlightMapper/Flight.info</t>
         </is>
       </c>
       <c r="N66" t="inlineStr">
         <is>
-          <t>https://booking.evaair.com/flyeva/eva/b2c/flight-schedules.aspx?lang=en-global</t>
+          <t>https://info.flightmapper.net/flight/EVA_Air_BR_716</t>
         </is>
       </c>
       <c r="O66" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="P66" t="inlineStr">
         <is>
-          <t>Cross-checked with FlightMapper route page; final EVA query should be re-run.</t>
+          <t>Confirmed for 2026 summer public schedule.</t>
         </is>
       </c>
     </row>
@@ -5868,22 +5868,22 @@
       </c>
       <c r="M67" t="inlineStr">
         <is>
-          <t>EVA Air official timetable page plus route-level cross-check</t>
+          <t>EVA Air official timetable page, cross-checked with FlightMapper/Flight.info</t>
         </is>
       </c>
       <c r="N67" t="inlineStr">
         <is>
-          <t>https://booking.evaair.com/flyeva/eva/b2c/flight-schedules.aspx?lang=en-global</t>
+          <t>https://info.flightmapper.net/flight/EVA_Air_BR_716</t>
         </is>
       </c>
       <c r="O67" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="P67" t="inlineStr">
         <is>
-          <t>Cross-checked with FlightMapper route page; final EVA query should be re-run.</t>
+          <t>Confirmed for 2026 summer public schedule.</t>
         </is>
       </c>
     </row>
@@ -5950,22 +5950,22 @@
       </c>
       <c r="M68" t="inlineStr">
         <is>
-          <t>EVA Air official timetable page plus route-level cross-check</t>
+          <t>EVA Air official timetable page, cross-checked with FlightMapper/Flight.info</t>
         </is>
       </c>
       <c r="N68" t="inlineStr">
         <is>
-          <t>https://booking.evaair.com/flyeva/eva/b2c/flight-schedules.aspx?lang=en-global</t>
+          <t>https://info.flightmapper.net/flight/EVA_Air_BR_715</t>
         </is>
       </c>
       <c r="O68" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>Cross-checked with FlightMapper route page; final EVA query should be re-run.</t>
+          <t>Confirmed for 2026 summer public schedule.</t>
         </is>
       </c>
     </row>
@@ -6032,22 +6032,22 @@
       </c>
       <c r="M69" t="inlineStr">
         <is>
-          <t>EVA Air official timetable page plus route-level cross-check</t>
+          <t>EVA Air official timetable page, cross-checked with FlightMapper/Flight.info</t>
         </is>
       </c>
       <c r="N69" t="inlineStr">
         <is>
-          <t>https://booking.evaair.com/flyeva/eva/b2c/flight-schedules.aspx?lang=en-global</t>
+          <t>https://info.flightmapper.net/flight/EVA_Air_BR_715</t>
         </is>
       </c>
       <c r="O69" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>Cross-checked with FlightMapper route page; final EVA query should be re-run.</t>
+          <t>Confirmed for 2026 summer public schedule.</t>
         </is>
       </c>
     </row>
@@ -6059,12 +6059,12 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>BR708</t>
+          <t>BR715</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>CAN</t>
+          <t>PEK</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -6074,27 +6074,27 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Guangzhou</t>
+          <t>Beijing Capital</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>Mon,Fri,Sun</t>
+          <t>Mon,Fri</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>1***5*7</t>
+          <t>1***5**</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>13:10</t>
+          <t>20:45</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>15:20</t>
+          <t>23:55</t>
         </is>
       </c>
       <c r="J70" t="inlineStr">
@@ -6109,27 +6109,27 @@
       </c>
       <c r="L70" t="inlineStr">
         <is>
-          <t>789</t>
+          <t>333</t>
         </is>
       </c>
       <c r="M70" t="inlineStr">
         <is>
-          <t>EVA Air official timetable page plus route-level cross-check</t>
+          <t>EVA Air official timetable page, cross-checked with FlightMapper/Flight.info</t>
         </is>
       </c>
       <c r="N70" t="inlineStr">
         <is>
-          <t>https://booking.evaair.com/flyeva/eva/b2c/flight-schedules.aspx?lang=en-global</t>
+          <t>https://info.flightmapper.net/flight/EVA_Air_BR_715</t>
         </is>
       </c>
       <c r="O70" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="P70" t="inlineStr">
         <is>
-          <t>Cross-checked with FlightMapper route page; final EVA query should be re-run.</t>
+          <t>Added after 2026 summer schedule confirmation.</t>
         </is>
       </c>
     </row>
@@ -6141,42 +6141,42 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>BR765</t>
+          <t>BR708</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
+          <t>CAN</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
           <t>TPE</t>
         </is>
       </c>
-      <c r="D71" t="inlineStr">
-        <is>
-          <t>TFU</t>
-        </is>
-      </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Chengdu Tianfu</t>
+          <t>Guangzhou</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>Mon,Fri</t>
+          <t>Mon,Fri,Sun</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>1***5**</t>
+          <t>1***5*7</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>13:10</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>18:05</t>
+          <t>15:20</t>
         </is>
       </c>
       <c r="J71" t="inlineStr">
@@ -6191,27 +6191,27 @@
       </c>
       <c r="L71" t="inlineStr">
         <is>
-          <t>333</t>
+          <t>789</t>
         </is>
       </c>
       <c r="M71" t="inlineStr">
         <is>
-          <t>EVA Air official timetable page plus route-level cross-check</t>
+          <t>EVA Air official timetable page, cross-checked with FlightMapper/Flight.info</t>
         </is>
       </c>
       <c r="N71" t="inlineStr">
         <is>
-          <t>https://booking.evaair.com/flyeva/eva/b2c/flight-schedules.aspx?lang=en-global</t>
+          <t>https://info.flightmapper.net/flight/EVA_Air_BR_708</t>
         </is>
       </c>
       <c r="O71" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="P71" t="inlineStr">
         <is>
-          <t>Cross-checked with FlightMapper route page; final EVA query should be re-run.</t>
+          <t>Confirmed for 2026 summer public schedule.</t>
         </is>
       </c>
     </row>
@@ -6223,42 +6223,42 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>BR711</t>
+          <t>BR765</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>PVG</t>
+          <t>TPE</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>TPE</t>
+          <t>TFU</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Shanghai Pudong</t>
+          <t>Chengdu Tianfu</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>Mon,Tue,Wed,Thu,Fri,Sat,Sun</t>
+          <t>Mon,Fri</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>Daily</t>
+          <t>1***5**</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>13:10</t>
+          <t>14:30</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>15:05</t>
+          <t>18:05</t>
         </is>
       </c>
       <c r="J72" t="inlineStr">
@@ -6273,27 +6273,27 @@
       </c>
       <c r="L72" t="inlineStr">
         <is>
-          <t>77W</t>
+          <t>333</t>
         </is>
       </c>
       <c r="M72" t="inlineStr">
         <is>
-          <t>EVA Air official timetable page plus route-level cross-check</t>
+          <t>EVA Air official timetable page, cross-checked with FlightMapper/Flight.info</t>
         </is>
       </c>
       <c r="N72" t="inlineStr">
         <is>
-          <t>https://booking.evaair.com/flyeva/eva/b2c/flight-schedules.aspx?lang=en-global</t>
+          <t>https://info.flightmapper.net/flight/EVA_Air_BR_765</t>
         </is>
       </c>
       <c r="O72" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="P72" t="inlineStr">
         <is>
-          <t>Cross-checked with FlightMapper route page; final EVA query should be re-run.</t>
+          <t>Confirmed for 2026 summer public schedule.</t>
         </is>
       </c>
     </row>
@@ -6305,7 +6305,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>BR721</t>
+          <t>BR711</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -6335,12 +6335,12 @@
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>20:05</t>
+          <t>13:15</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>15:15</t>
         </is>
       </c>
       <c r="J73" t="inlineStr">
@@ -6355,54 +6355,54 @@
       </c>
       <c r="L73" t="inlineStr">
         <is>
-          <t>333</t>
+          <t>77W</t>
         </is>
       </c>
       <c r="M73" t="inlineStr">
         <is>
-          <t>EVA Air official timetable page plus route-level cross-check</t>
+          <t>EVA Air official timetable page, cross-checked with FlightMapper/Flight.info</t>
         </is>
       </c>
       <c r="N73" t="inlineStr">
         <is>
-          <t>https://booking.evaair.com/flyeva/eva/b2c/flight-schedules.aspx?lang=en-global</t>
+          <t>https://info.flightmapper.net/flight/EVA_Air_BR_711</t>
         </is>
       </c>
       <c r="O73" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="P73" t="inlineStr">
         <is>
-          <t>Cross-checked with FlightMapper route page; final EVA query should be re-run.</t>
+          <t>Time corrected after 2026 winter-forward schedule check.</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>FM</t>
+          <t>BR</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>FM802</t>
+          <t>BR721</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>TSA</t>
+          <t>PVG</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>SHA</t>
+          <t>TPE</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Shanghai Hongqiao</t>
+          <t>Shanghai Pudong</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -6417,12 +6417,12 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>12:05</t>
+          <t>20:05</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>13:40</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="J74" t="inlineStr">
@@ -6435,25 +6435,29 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="L74" t="inlineStr"/>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>333</t>
+        </is>
+      </c>
       <c r="M74" t="inlineStr">
         <is>
-          <t>China Eastern Taiwan timetable PDF</t>
+          <t>EVA Air official timetable page, cross-checked with FlightMapper/Flight.info</t>
         </is>
       </c>
       <c r="N74" t="inlineStr">
         <is>
-          <t>https://tw.ceair.com/newwebsite/tw/upload/China-Eastern-Airlines2018timetable.pdf</t>
+          <t>https://info.flightmapper.net/flight/EVA_Air_BR_721</t>
         </is>
       </c>
       <c r="O74" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="P74" t="inlineStr">
         <is>
-          <t>Official PDF table is older/undated for 2026; retained for review.</t>
+          <t>Confirmed for 2026 summer public schedule.</t>
         </is>
       </c>
     </row>
@@ -6465,7 +6469,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>FM820</t>
+          <t>FM802</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -6475,12 +6479,12 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>PVG</t>
+          <t>SHA</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Shanghai Pudong</t>
+          <t>Shanghai Hongqiao</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -6495,12 +6499,12 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
+          <t>12:05</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
           <t>13:40</t>
-        </is>
-      </c>
-      <c r="I75" t="inlineStr">
-        <is>
-          <t>15:35</t>
         </is>
       </c>
       <c r="J75" t="inlineStr">
@@ -6516,7 +6520,7 @@
       <c r="L75" t="inlineStr"/>
       <c r="M75" t="inlineStr">
         <is>
-          <t>China Eastern Taiwan timetable PDF</t>
+          <t>China Eastern Taiwan timetable PDF, cross-checked with public flight schedule pages</t>
         </is>
       </c>
       <c r="N75" t="inlineStr">
@@ -6526,24 +6530,24 @@
       </c>
       <c r="O75" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="P75" t="inlineStr">
         <is>
-          <t>Official PDF table is older/undated for 2026; retained for review.</t>
+          <t>Confirmed against China Eastern Taiwan timetable PDF.</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>MU</t>
+          <t>FM</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>MU5098</t>
+          <t>FM820</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -6563,22 +6567,22 @@
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>Mon,Tue,Wed,Thu,Sat,Sun</t>
+          <t>Mon,Tue,Wed,Thu,Fri,Sat,Sun</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>1234*67</t>
+          <t>Daily</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>17:15</t>
+          <t>13:40</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>18:55</t>
+          <t>15:35</t>
         </is>
       </c>
       <c r="J76" t="inlineStr">
@@ -6594,7 +6598,7 @@
       <c r="L76" t="inlineStr"/>
       <c r="M76" t="inlineStr">
         <is>
-          <t>China Eastern Taiwan timetable PDF</t>
+          <t>China Eastern Taiwan timetable PDF, cross-checked with public flight schedule pages</t>
         </is>
       </c>
       <c r="N76" t="inlineStr">
@@ -6604,12 +6608,12 @@
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="P76" t="inlineStr">
         <is>
-          <t>Official PDF table is older/undated for 2026; retained for review.</t>
+          <t>Confirmed against China Eastern Taiwan timetable PDF.</t>
         </is>
       </c>
     </row>
@@ -6621,42 +6625,42 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>MU2942</t>
+          <t>MU5098</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>RMQ</t>
+          <t>TSA</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>NKG</t>
+          <t>PVG</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Nanjing</t>
+          <t>Shanghai Pudong</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>Sat</t>
+          <t>Mon,Tue,Wed,Thu,Sat,Sun</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>*****6*</t>
+          <t>1234*67</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>17:15</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>13:10</t>
+          <t>18:55</t>
         </is>
       </c>
       <c r="J77" t="inlineStr">
@@ -6672,7 +6676,7 @@
       <c r="L77" t="inlineStr"/>
       <c r="M77" t="inlineStr">
         <is>
-          <t>China Eastern Taiwan timetable PDF</t>
+          <t>China Eastern Taiwan timetable PDF, cross-checked with public flight schedule pages</t>
         </is>
       </c>
       <c r="N77" t="inlineStr">
@@ -6682,12 +6686,12 @@
       </c>
       <c r="O77" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="P77" t="inlineStr">
         <is>
-          <t>Official PDF table is older/undated for 2026; retained for review.</t>
+          <t>Confirmed against China Eastern Taiwan timetable PDF.</t>
         </is>
       </c>
     </row>
@@ -6699,42 +6703,42 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>MU2662</t>
+          <t>MU2942</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>KHH</t>
+          <t>RMQ</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>NCH</t>
+          <t>NKG</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Nanchang</t>
+          <t>Nanjing</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>Fri,Sun</t>
+          <t>Sat</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>****5*7</t>
+          <t>*****6*</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>18:15</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>13:10</t>
         </is>
       </c>
       <c r="J78" t="inlineStr">
@@ -6750,7 +6754,7 @@
       <c r="L78" t="inlineStr"/>
       <c r="M78" t="inlineStr">
         <is>
-          <t>China Eastern Taiwan timetable PDF</t>
+          <t>China Eastern Taiwan timetable PDF, cross-checked with public flight schedule pages</t>
         </is>
       </c>
       <c r="N78" t="inlineStr">
@@ -6760,12 +6764,12 @@
       </c>
       <c r="O78" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="P78" t="inlineStr">
         <is>
-          <t>Official PDF table is older/undated for 2026; retained for review.</t>
+          <t>Confirmed against China Eastern Taiwan timetable PDF.</t>
         </is>
       </c>
     </row>
@@ -6777,7 +6781,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>MU2722</t>
+          <t>MU2662</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -6787,32 +6791,32 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>WUX</t>
+          <t>NCH</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Wuxi</t>
+          <t>Nanchang</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>Wed,Sun</t>
+          <t>Fri,Sun</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>**3***7</t>
+          <t>****5*7</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>17:30</t>
+          <t>18:15</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>20:05</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="J79" t="inlineStr">
@@ -6828,7 +6832,7 @@
       <c r="L79" t="inlineStr"/>
       <c r="M79" t="inlineStr">
         <is>
-          <t>China Eastern Taiwan timetable PDF</t>
+          <t>China Eastern Taiwan timetable PDF, cross-checked with public flight schedule pages</t>
         </is>
       </c>
       <c r="N79" t="inlineStr">
@@ -6838,59 +6842,59 @@
       </c>
       <c r="O79" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="P79" t="inlineStr">
         <is>
-          <t>Regular charter note in source; reconfirm before use.</t>
+          <t>Confirmed against China Eastern Taiwan timetable PDF.</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>FM</t>
+          <t>MU</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>FM851</t>
+          <t>MU2722</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>SHA</t>
+          <t>KHH</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>TSA</t>
+          <t>WUX</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Shanghai Hongqiao</t>
+          <t>Wuxi</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>Tue,Fri,Sun</t>
+          <t>Wed,Sun</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>*2**5*7</t>
+          <t>**3***7</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>09:10</t>
+          <t>17:30</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>10:45</t>
+          <t>20:05</t>
         </is>
       </c>
       <c r="J80" t="inlineStr">
@@ -6906,7 +6910,7 @@
       <c r="L80" t="inlineStr"/>
       <c r="M80" t="inlineStr">
         <is>
-          <t>China Eastern Taiwan timetable PDF</t>
+          <t>China Eastern Taiwan timetable PDF, cross-checked with public flight schedule pages</t>
         </is>
       </c>
       <c r="N80" t="inlineStr">
@@ -6916,29 +6920,29 @@
       </c>
       <c r="O80" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="P80" t="inlineStr">
         <is>
-          <t>Official PDF table is older/undated for 2026; retained for review.</t>
+          <t>Confirmed against China Eastern Taiwan timetable PDF; source marks this as regular charter.</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>MU</t>
+          <t>FM</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>MU5097</t>
+          <t>FM851</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>PVG</t>
+          <t>SHA</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -6948,27 +6952,27 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Shanghai Pudong</t>
+          <t>Shanghai Hongqiao</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>Mon,Tue,Wed,Thu,Fri,Sat,Sun</t>
+          <t>Tue,Fri,Sun</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>Daily</t>
+          <t>*2**5*7</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>14:20</t>
+          <t>09:10</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>16:15</t>
+          <t>10:45</t>
         </is>
       </c>
       <c r="J81" t="inlineStr">
@@ -6984,7 +6988,7 @@
       <c r="L81" t="inlineStr"/>
       <c r="M81" t="inlineStr">
         <is>
-          <t>China Eastern Taiwan timetable PDF</t>
+          <t>China Eastern Taiwan timetable PDF, cross-checked with public flight schedule pages</t>
         </is>
       </c>
       <c r="N81" t="inlineStr">
@@ -6994,29 +6998,29 @@
       </c>
       <c r="O81" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="P81" t="inlineStr">
         <is>
-          <t>Official PDF table is older/undated for 2026; retained for review.</t>
+          <t>Confirmed against China Eastern Taiwan timetable PDF.</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>FM</t>
+          <t>MU</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>FM801</t>
+          <t>MU5097</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>SHA</t>
+          <t>PVG</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -7026,7 +7030,7 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Shanghai Hongqiao</t>
+          <t>Shanghai Pudong</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -7041,12 +7045,12 @@
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>09:25</t>
+          <t>14:20</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>11:05</t>
+          <t>16:15</t>
         </is>
       </c>
       <c r="J82" t="inlineStr">
@@ -7062,7 +7066,7 @@
       <c r="L82" t="inlineStr"/>
       <c r="M82" t="inlineStr">
         <is>
-          <t>China Eastern Taiwan timetable PDF</t>
+          <t>China Eastern Taiwan timetable PDF, cross-checked with public flight schedule pages</t>
         </is>
       </c>
       <c r="N82" t="inlineStr">
@@ -7072,12 +7076,12 @@
       </c>
       <c r="O82" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="P82" t="inlineStr">
         <is>
-          <t>Official PDF table is older/undated for 2026; retained for review.</t>
+          <t>Confirmed against China Eastern Taiwan timetable PDF.</t>
         </is>
       </c>
     </row>
@@ -7089,12 +7093,12 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>FM819</t>
+          <t>FM801</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>PVG</t>
+          <t>SHA</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -7104,27 +7108,27 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Shanghai Pudong</t>
+          <t>Shanghai Hongqiao</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>Mon,Wed,Sat</t>
+          <t>Mon,Tue,Wed,Thu,Fri,Sat,Sun</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>1*3**6*</t>
+          <t>Daily</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
         <is>
+          <t>09:25</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
           <t>11:05</t>
-        </is>
-      </c>
-      <c r="I83" t="inlineStr">
-        <is>
-          <t>12:40</t>
         </is>
       </c>
       <c r="J83" t="inlineStr">
@@ -7140,7 +7144,7 @@
       <c r="L83" t="inlineStr"/>
       <c r="M83" t="inlineStr">
         <is>
-          <t>China Eastern Taiwan timetable PDF</t>
+          <t>China Eastern Taiwan timetable PDF, cross-checked with public flight schedule pages</t>
         </is>
       </c>
       <c r="N83" t="inlineStr">
@@ -7150,59 +7154,59 @@
       </c>
       <c r="O83" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="P83" t="inlineStr">
         <is>
-          <t>Official PDF table is older/undated for 2026; retained for review.</t>
+          <t>Confirmed against China Eastern Taiwan timetable PDF.</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>MU</t>
+          <t>FM</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>MU2941</t>
+          <t>FM819</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>NKG</t>
+          <t>PVG</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>RMQ</t>
+          <t>TSA</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Nanjing</t>
+          <t>Shanghai Pudong</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>Sat</t>
+          <t>Mon,Wed,Sat</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>*****6*</t>
+          <t>1*3**6*</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>08:00</t>
+          <t>11:05</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>10:10</t>
+          <t>12:40</t>
         </is>
       </c>
       <c r="J84" t="inlineStr">
@@ -7218,7 +7222,7 @@
       <c r="L84" t="inlineStr"/>
       <c r="M84" t="inlineStr">
         <is>
-          <t>China Eastern Taiwan timetable PDF</t>
+          <t>China Eastern Taiwan timetable PDF, cross-checked with public flight schedule pages</t>
         </is>
       </c>
       <c r="N84" t="inlineStr">
@@ -7228,12 +7232,12 @@
       </c>
       <c r="O84" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="P84" t="inlineStr">
         <is>
-          <t>Official PDF table is older/undated for 2026; retained for review.</t>
+          <t>Confirmed against China Eastern Taiwan timetable PDF.</t>
         </is>
       </c>
     </row>
@@ -7245,42 +7249,42 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>MU2661</t>
+          <t>MU2941</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>NCH</t>
+          <t>NKG</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>KHH</t>
+          <t>RMQ</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Nanchang</t>
+          <t>Nanjing</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>Fri,Sun</t>
+          <t>Sat</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>****5*7</t>
+          <t>*****6*</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>17:15</t>
+          <t>10:10</t>
         </is>
       </c>
       <c r="J85" t="inlineStr">
@@ -7296,7 +7300,7 @@
       <c r="L85" t="inlineStr"/>
       <c r="M85" t="inlineStr">
         <is>
-          <t>China Eastern Taiwan timetable PDF</t>
+          <t>China Eastern Taiwan timetable PDF, cross-checked with public flight schedule pages</t>
         </is>
       </c>
       <c r="N85" t="inlineStr">
@@ -7306,12 +7310,12 @@
       </c>
       <c r="O85" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="P85" t="inlineStr">
         <is>
-          <t>Official PDF table is older/undated for 2026; retained for review.</t>
+          <t>Confirmed against China Eastern Taiwan timetable PDF.</t>
         </is>
       </c>
     </row>
@@ -7323,12 +7327,12 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>MU2721</t>
+          <t>MU2661</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>WUX</t>
+          <t>NCH</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -7338,27 +7342,27 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Wuxi</t>
+          <t>Nanchang</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>Wed,Sun</t>
+          <t>Fri,Sun</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>**3***7</t>
+          <t>****5*7</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>14:05</t>
+          <t>14:30</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>17:15</t>
         </is>
       </c>
       <c r="J86" t="inlineStr">
@@ -7374,7 +7378,7 @@
       <c r="L86" t="inlineStr"/>
       <c r="M86" t="inlineStr">
         <is>
-          <t>China Eastern Taiwan timetable PDF</t>
+          <t>China Eastern Taiwan timetable PDF, cross-checked with public flight schedule pages</t>
         </is>
       </c>
       <c r="N86" t="inlineStr">
@@ -7384,12 +7388,12 @@
       </c>
       <c r="O86" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="P86" t="inlineStr">
         <is>
-          <t>Regular charter note in source; reconfirm before use.</t>
+          <t>Confirmed against China Eastern Taiwan timetable PDF.</t>
         </is>
       </c>
     </row>
@@ -7401,42 +7405,42 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>MU5008</t>
+          <t>MU2721</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>TPE</t>
+          <t>WUX</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>PVG</t>
+          <t>KHH</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Shanghai Pudong</t>
+          <t>Wuxi</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>Mon,Tue,Wed,Thu,Fri,Sat,Sun</t>
+          <t>Wed,Sun</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>Daily</t>
+          <t>**3***7</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>15:30</t>
+          <t>14:05</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>17:20</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="J87" t="inlineStr">
@@ -7452,7 +7456,7 @@
       <c r="L87" t="inlineStr"/>
       <c r="M87" t="inlineStr">
         <is>
-          <t>China Eastern Taiwan timetable PDF</t>
+          <t>China Eastern Taiwan timetable PDF, cross-checked with public flight schedule pages</t>
         </is>
       </c>
       <c r="N87" t="inlineStr">
@@ -7462,12 +7466,12 @@
       </c>
       <c r="O87" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="P87" t="inlineStr">
         <is>
-          <t>Official PDF table is older/undated for 2026; retained for review.</t>
+          <t>Confirmed against China Eastern Taiwan timetable PDF; source marks this as regular charter.</t>
         </is>
       </c>
     </row>
@@ -7479,7 +7483,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>MU5006</t>
+          <t>MU5008</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -7499,22 +7503,22 @@
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>Mon,Thu,Fri,Sat,Sun</t>
+          <t>Mon,Tue,Wed,Thu,Fri,Sat,Sun</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>1**4567</t>
+          <t>Daily</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>18:40</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>20:35</t>
+          <t>17:20</t>
         </is>
       </c>
       <c r="J88" t="inlineStr">
@@ -7530,7 +7534,7 @@
       <c r="L88" t="inlineStr"/>
       <c r="M88" t="inlineStr">
         <is>
-          <t>China Eastern Taiwan timetable PDF</t>
+          <t>China Eastern Taiwan timetable PDF, cross-checked with public flight schedule pages</t>
         </is>
       </c>
       <c r="N88" t="inlineStr">
@@ -7540,12 +7544,12 @@
       </c>
       <c r="O88" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="P88" t="inlineStr">
         <is>
-          <t>Official PDF table is older/undated for 2026; retained for review.</t>
+          <t>Confirmed against China Eastern Taiwan timetable PDF; public schedule pages show later seasonal variants.</t>
         </is>
       </c>
     </row>
@@ -7557,7 +7561,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>MU2088</t>
+          <t>MU5006</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -7567,22 +7571,22 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>WUH</t>
+          <t>PVG</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Wuhan</t>
+          <t>Shanghai Pudong</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>Mon</t>
+          <t>Mon,Thu,Fri,Sat,Sun</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>1******</t>
+          <t>1**4567</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
@@ -7592,7 +7596,7 @@
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>20:35</t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
@@ -7608,7 +7612,7 @@
       <c r="L89" t="inlineStr"/>
       <c r="M89" t="inlineStr">
         <is>
-          <t>China Eastern Taiwan timetable PDF</t>
+          <t>China Eastern Taiwan timetable PDF, cross-checked with public flight schedule pages</t>
         </is>
       </c>
       <c r="N89" t="inlineStr">
@@ -7618,12 +7622,12 @@
       </c>
       <c r="O89" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="P89" t="inlineStr">
         <is>
-          <t>Official PDF table is older/undated for 2026; retained for review.</t>
+          <t>Confirmed against China Eastern Taiwan timetable PDF.</t>
         </is>
       </c>
     </row>
@@ -7635,7 +7639,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>MU2010</t>
+          <t>MU2088</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -7645,32 +7649,32 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>NGB</t>
+          <t>WUH</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Ningbo</t>
+          <t>Wuhan</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>Mon,Wed,Thu,Fri</t>
+          <t>Mon</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>1*345**</t>
+          <t>1******</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>11:15</t>
+          <t>18:40</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>12:55</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="J90" t="inlineStr">
@@ -7686,7 +7690,7 @@
       <c r="L90" t="inlineStr"/>
       <c r="M90" t="inlineStr">
         <is>
-          <t>China Eastern Taiwan timetable PDF</t>
+          <t>China Eastern Taiwan timetable PDF, cross-checked with public flight schedule pages</t>
         </is>
       </c>
       <c r="N90" t="inlineStr">
@@ -7696,12 +7700,12 @@
       </c>
       <c r="O90" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="P90" t="inlineStr">
         <is>
-          <t>Official PDF table is older/undated for 2026; retained for review.</t>
+          <t>Confirmed against China Eastern Taiwan timetable PDF.</t>
         </is>
       </c>
     </row>
@@ -7713,7 +7717,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>MU2982</t>
+          <t>MU2010</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -7723,32 +7727,32 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>NKG</t>
+          <t>NGB</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Nanjing</t>
+          <t>Ningbo</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>Mon</t>
+          <t>Mon,Wed,Thu,Fri</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>1******</t>
+          <t>1*345**</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>10:50</t>
+          <t>11:15</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>13:05</t>
+          <t>12:55</t>
         </is>
       </c>
       <c r="J91" t="inlineStr">
@@ -7764,7 +7768,7 @@
       <c r="L91" t="inlineStr"/>
       <c r="M91" t="inlineStr">
         <is>
-          <t>China Eastern Taiwan timetable PDF</t>
+          <t>China Eastern Taiwan timetable PDF, cross-checked with public flight schedule pages</t>
         </is>
       </c>
       <c r="N91" t="inlineStr">
@@ -7774,12 +7778,12 @@
       </c>
       <c r="O91" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="P91" t="inlineStr">
         <is>
-          <t>Official PDF table is older/undated for 2026; retained for review.</t>
+          <t>Confirmed against China Eastern Taiwan timetable PDF.</t>
         </is>
       </c>
     </row>
@@ -7791,7 +7795,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>MU5002</t>
+          <t>MU2982</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -7811,22 +7815,22 @@
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>Mon,Tue,Wed,Thu,Fri,Sat,Sun</t>
+          <t>Mon</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>Daily</t>
+          <t>1******</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>17:20</t>
+          <t>10:50</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>19:30</t>
+          <t>13:05</t>
         </is>
       </c>
       <c r="J92" t="inlineStr">
@@ -7842,7 +7846,7 @@
       <c r="L92" t="inlineStr"/>
       <c r="M92" t="inlineStr">
         <is>
-          <t>China Eastern Taiwan timetable PDF</t>
+          <t>China Eastern Taiwan timetable PDF, cross-checked with public flight schedule pages</t>
         </is>
       </c>
       <c r="N92" t="inlineStr">
@@ -7852,12 +7856,12 @@
       </c>
       <c r="O92" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="P92" t="inlineStr">
         <is>
-          <t>Official PDF table is older/undated for 2026; retained for review.</t>
+          <t>Confirmed against China Eastern Taiwan timetable PDF.</t>
         </is>
       </c>
     </row>
@@ -7869,7 +7873,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>MU2042</t>
+          <t>MU5002</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -7879,32 +7883,32 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>TAO</t>
+          <t>NKG</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Qingdao</t>
+          <t>Nanjing</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>Fri</t>
+          <t>Mon,Tue,Wed,Thu,Fri,Sat,Sun</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>****5**</t>
+          <t>Daily</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>17:20</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>15:30</t>
+          <t>19:30</t>
         </is>
       </c>
       <c r="J93" t="inlineStr">
@@ -7920,7 +7924,7 @@
       <c r="L93" t="inlineStr"/>
       <c r="M93" t="inlineStr">
         <is>
-          <t>China Eastern Taiwan timetable PDF</t>
+          <t>China Eastern Taiwan timetable PDF, cross-checked with public flight schedule pages</t>
         </is>
       </c>
       <c r="N93" t="inlineStr">
@@ -7930,12 +7934,12 @@
       </c>
       <c r="O93" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="P93" t="inlineStr">
         <is>
-          <t>Official PDF table is older/undated for 2026; retained for review.</t>
+          <t>Confirmed against China Eastern Taiwan timetable PDF.</t>
         </is>
       </c>
     </row>
@@ -7947,42 +7951,42 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>MU2047</t>
+          <t>MU2042</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>NCH</t>
+          <t>TPE</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>TPE</t>
+          <t>TAO</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Nanchang</t>
+          <t>Qingdao</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>Mon,Thu,Fri,Sat</t>
+          <t>Fri</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>1**456*</t>
+          <t>****5**</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>08:35</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>10:45</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="J94" t="inlineStr">
@@ -7998,7 +8002,7 @@
       <c r="L94" t="inlineStr"/>
       <c r="M94" t="inlineStr">
         <is>
-          <t>China Eastern Taiwan timetable PDF</t>
+          <t>China Eastern Taiwan timetable PDF, cross-checked with public flight schedule pages</t>
         </is>
       </c>
       <c r="N94" t="inlineStr">
@@ -8008,12 +8012,12 @@
       </c>
       <c r="O94" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="P94" t="inlineStr">
         <is>
-          <t>Official PDF table is older/undated for 2026; retained for review.</t>
+          <t>Confirmed against China Eastern Taiwan timetable PDF.</t>
         </is>
       </c>
     </row>
@@ -8025,12 +8029,12 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>MU2041</t>
+          <t>MU2047</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>TAO</t>
+          <t>NCH</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -8040,27 +8044,27 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Qingdao</t>
+          <t>Nanchang</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>Fri</t>
+          <t>Mon,Thu,Fri,Sat</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>****5**</t>
+          <t>1**456*</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>08:50</t>
+          <t>08:35</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>11:35</t>
+          <t>10:45</t>
         </is>
       </c>
       <c r="J95" t="inlineStr">
@@ -8076,7 +8080,7 @@
       <c r="L95" t="inlineStr"/>
       <c r="M95" t="inlineStr">
         <is>
-          <t>China Eastern Taiwan timetable PDF</t>
+          <t>China Eastern Taiwan timetable PDF, cross-checked with public flight schedule pages</t>
         </is>
       </c>
       <c r="N95" t="inlineStr">
@@ -8086,12 +8090,12 @@
       </c>
       <c r="O95" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="P95" t="inlineStr">
         <is>
-          <t>Official PDF table is older/undated for 2026; retained for review.</t>
+          <t>Confirmed against China Eastern Taiwan timetable PDF.</t>
         </is>
       </c>
     </row>
@@ -8103,12 +8107,12 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>MU2087</t>
+          <t>MU2041</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>WUH</t>
+          <t>TAO</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -8118,27 +8122,27 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Wuhan</t>
+          <t>Qingdao</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>Mon</t>
+          <t>Fri</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>1******</t>
+          <t>****5**</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>14:55</t>
+          <t>08:50</t>
         </is>
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>17:30</t>
+          <t>11:35</t>
         </is>
       </c>
       <c r="J96" t="inlineStr">
@@ -8154,7 +8158,7 @@
       <c r="L96" t="inlineStr"/>
       <c r="M96" t="inlineStr">
         <is>
-          <t>China Eastern Taiwan timetable PDF</t>
+          <t>China Eastern Taiwan timetable PDF, cross-checked with public flight schedule pages</t>
         </is>
       </c>
       <c r="N96" t="inlineStr">
@@ -8164,12 +8168,12 @@
       </c>
       <c r="O96" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="P96" t="inlineStr">
         <is>
-          <t>Official PDF table is older/undated for 2026; retained for review.</t>
+          <t>Confirmed against China Eastern Taiwan timetable PDF.</t>
         </is>
       </c>
     </row>
@@ -8181,12 +8185,12 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>MU2981</t>
+          <t>MU2087</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>NKG</t>
+          <t>WUH</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -8196,27 +8200,27 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Nanjing</t>
+          <t>Wuhan</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>Mon,Tue,Wed,Thu,Fri,Sat,Sun</t>
+          <t>Mon</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>Daily</t>
+          <t>1******</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>07:45</t>
+          <t>14:55</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>09:50</t>
+          <t>17:30</t>
         </is>
       </c>
       <c r="J97" t="inlineStr">
@@ -8232,7 +8236,7 @@
       <c r="L97" t="inlineStr"/>
       <c r="M97" t="inlineStr">
         <is>
-          <t>China Eastern Taiwan timetable PDF</t>
+          <t>China Eastern Taiwan timetable PDF, cross-checked with public flight schedule pages</t>
         </is>
       </c>
       <c r="N97" t="inlineStr">
@@ -8242,12 +8246,12 @@
       </c>
       <c r="O97" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="P97" t="inlineStr">
         <is>
-          <t>Official PDF table is older/undated for 2026; retained for review.</t>
+          <t>Confirmed against China Eastern Taiwan timetable PDF.</t>
         </is>
       </c>
     </row>
@@ -8259,7 +8263,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>MU5001</t>
+          <t>MU2981</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -8289,12 +8293,12 @@
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>07:45</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>16:25</t>
+          <t>09:50</t>
         </is>
       </c>
       <c r="J98" t="inlineStr">
@@ -8310,7 +8314,7 @@
       <c r="L98" t="inlineStr"/>
       <c r="M98" t="inlineStr">
         <is>
-          <t>China Eastern Taiwan timetable PDF</t>
+          <t>China Eastern Taiwan timetable PDF, cross-checked with public flight schedule pages</t>
         </is>
       </c>
       <c r="N98" t="inlineStr">
@@ -8320,12 +8324,12 @@
       </c>
       <c r="O98" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="P98" t="inlineStr">
         <is>
-          <t>Official PDF table is older/undated for 2026; retained for review.</t>
+          <t>Confirmed against China Eastern Taiwan timetable PDF.</t>
         </is>
       </c>
     </row>
@@ -8337,12 +8341,12 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>MU5007</t>
+          <t>MU5001</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>PVG</t>
+          <t>NKG</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -8352,7 +8356,7 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Shanghai Pudong</t>
+          <t>Nanjing</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
@@ -8367,12 +8371,12 @@
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>12:25</t>
+          <t>14:30</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>14:25</t>
+          <t>16:25</t>
         </is>
       </c>
       <c r="J99" t="inlineStr">
@@ -8388,7 +8392,7 @@
       <c r="L99" t="inlineStr"/>
       <c r="M99" t="inlineStr">
         <is>
-          <t>China Eastern Taiwan timetable PDF</t>
+          <t>China Eastern Taiwan timetable PDF, cross-checked with public flight schedule pages</t>
         </is>
       </c>
       <c r="N99" t="inlineStr">
@@ -8398,12 +8402,12 @@
       </c>
       <c r="O99" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="P99" t="inlineStr">
         <is>
-          <t>Official PDF table is older/undated for 2026; retained for review.</t>
+          <t>Confirmed against China Eastern Taiwan timetable PDF.</t>
         </is>
       </c>
     </row>
@@ -8415,7 +8419,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>MU5005</t>
+          <t>MU5007</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -8435,22 +8439,22 @@
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>Mon,Thu,Fri,Sat,Sun</t>
+          <t>Mon,Tue,Wed,Thu,Fri,Sat,Sun</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>1**4567</t>
+          <t>Daily</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>19:50</t>
+          <t>12:25</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>21:40</t>
+          <t>14:25</t>
         </is>
       </c>
       <c r="J100" t="inlineStr">
@@ -8466,7 +8470,7 @@
       <c r="L100" t="inlineStr"/>
       <c r="M100" t="inlineStr">
         <is>
-          <t>China Eastern Taiwan timetable PDF</t>
+          <t>China Eastern Taiwan timetable PDF, cross-checked with public flight schedule pages</t>
         </is>
       </c>
       <c r="N100" t="inlineStr">
@@ -8476,12 +8480,12 @@
       </c>
       <c r="O100" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="P100" t="inlineStr">
         <is>
-          <t>Official PDF table is older/undated for 2026; retained for review.</t>
+          <t>Confirmed against China Eastern Taiwan timetable PDF.</t>
         </is>
       </c>
     </row>
@@ -8493,12 +8497,12 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>MU2009</t>
+          <t>MU5005</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>NGB</t>
+          <t>PVG</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -8508,27 +8512,27 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Ningbo</t>
+          <t>Shanghai Pudong</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>Mon,Tue,Wed,Thu,Fri,Sat,Sun</t>
+          <t>Mon,Thu,Fri,Sat,Sun</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>Daily</t>
+          <t>1**4567</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>08:40</t>
+          <t>19:50</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>10:20</t>
+          <t>21:40</t>
         </is>
       </c>
       <c r="J101" t="inlineStr">
@@ -8544,7 +8548,7 @@
       <c r="L101" t="inlineStr"/>
       <c r="M101" t="inlineStr">
         <is>
-          <t>China Eastern Taiwan timetable PDF</t>
+          <t>China Eastern Taiwan timetable PDF, cross-checked with public flight schedule pages</t>
         </is>
       </c>
       <c r="N101" t="inlineStr">
@@ -8554,17 +8558,95 @@
       </c>
       <c r="O101" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="P101" t="inlineStr">
         <is>
-          <t>Official PDF table is older/undated for 2026; retained for review.</t>
+          <t>Confirmed against China Eastern Taiwan timetable PDF.</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>MU2009</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>NGB</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>TPE</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>Ningbo</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>Mon,Tue,Wed,Thu,Fri,Sat,Sun</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>Daily</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>08:40</t>
+        </is>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>10:20</t>
+        </is>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="K102" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="L102" t="inlineStr"/>
+      <c r="M102" t="inlineStr">
+        <is>
+          <t>China Eastern Taiwan timetable PDF, cross-checked with public flight schedule pages</t>
+        </is>
+      </c>
+      <c r="N102" t="inlineStr">
+        <is>
+          <t>https://tw.ceair.com/newwebsite/tw/upload/China-Eastern-Airlines2018timetable.pdf</t>
+        </is>
+      </c>
+      <c r="O102" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="P102" t="inlineStr">
+        <is>
+          <t>Confirmed against China Eastern Taiwan timetable PDF.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P101"/>
+  <autoFilter ref="A1:P102"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -8660,10 +8742,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C4" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -9074,7 +9156,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C18" t="n">
         <v>6</v>

</xml_diff>